<commit_message>
Update docs , add gitIgnore
</commit_message>
<xml_diff>
--- a/docs/planning/planning.xlsx
+++ b/docs/planning/planning.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/congdinh/Library/Mobile Documents/com~apple~CloudDocs/works/mentor/classes/HN24_FRF_FJB_03/Mock/ims-ninja/docs/planning/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CS\IMS-Mock-Project\ims\docs\planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE5C7867-00B7-4045-8D5F-F9DEC8F40FDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BBB0D11-1A34-40D3-A3E8-A47370928710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2860" windowWidth="28480" windowHeight="17000" xr2:uid="{C19F09B8-63BC-4CE7-BFBE-7F2585E3E38B}"/>
+    <workbookView xWindow="12946" yWindow="0" windowWidth="13232" windowHeight="14047" xr2:uid="{C19F09B8-63BC-4CE7-BFBE-7F2585E3E38B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>#</t>
   </si>
@@ -63,67 +63,6 @@
   </si>
   <si>
     <t>Module Desc</t>
-  </si>
-  <si>
-    <t>Candidate</t>
-  </si>
-  <si>
-    <t>Job</t>
-  </si>
-  <si>
-    <t>Interview</t>
-  </si>
-  <si>
-    <t>Offer</t>
-  </si>
-  <si>
-    <t>Auth + User</t>
-  </si>
-  <si>
-    <t>UC05 View Candidate List
-UC06: Create new Candidate
-UC08: Edit Candidate Information
-UC09: Delete Candidate</t>
-  </si>
-  <si>
-    <t>UC23: View offer list
-UC24 Create new offer
-UC25 Edit offer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UC16 View interview schedule
-UC17 Create interview schedule
-UC20 Edit interview
-</t>
-  </si>
-  <si>
-    <t>UC12 Create Job
-UC11 View job list
-UC14 Edit job
-UC15 Delete job</t>
-  </si>
-  <si>
-    <t>UC32 View user list
-UC33 Create new user
-UC35 Edit user</t>
-  </si>
-  <si>
-    <t>14h 30/12/2024</t>
-  </si>
-  <si>
-    <t>14h 30/12/2025</t>
-  </si>
-  <si>
-    <t>14h 30/12/2026</t>
-  </si>
-  <si>
-    <t>14h 30/12/2028</t>
-  </si>
-  <si>
-    <t>14h 30/12/2029</t>
-  </si>
-  <si>
-    <t>PENDING</t>
   </si>
 </sst>
 </file>
@@ -641,19 +580,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{612C22F7-DEDF-4EDF-AEE8-648848F99654}">
   <dimension ref="A1:I8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.3"/>
   <cols>
     <col min="2" max="2" width="19.5" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="27.33203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="27.375" customWidth="1"/>
+    <col min="5" max="5" width="16.875" customWidth="1"/>
     <col min="6" max="6" width="17.5" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.6640625" customWidth="1"/>
-    <col min="9" max="9" width="20.1640625" customWidth="1"/>
+    <col min="7" max="7" width="16.375" customWidth="1"/>
+    <col min="8" max="8" width="15.625" customWidth="1"/>
+    <col min="9" max="9" width="20.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16">
+    <row r="1" spans="1:9" ht="16.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -682,66 +621,40 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="64">
+    <row r="2" spans="1:9">
       <c r="A2" s="15">
         <v>0</v>
       </c>
-      <c r="B2" s="15">
-        <v>1</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>14</v>
-      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="9"/>
       <c r="E2" s="8"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" s="13" t="s">
-        <v>24</v>
-      </c>
+      <c r="H2" s="12"/>
+      <c r="I2" s="13"/>
     </row>
-    <row r="3" spans="1:9" ht="48">
+    <row r="3" spans="1:9">
       <c r="A3" s="16"/>
       <c r="B3" s="16"/>
-      <c r="C3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>15</v>
-      </c>
+      <c r="C3" s="6"/>
+      <c r="D3" s="10"/>
       <c r="E3" s="8"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="13" t="s">
-        <v>24</v>
-      </c>
+      <c r="H3" s="12"/>
+      <c r="I3" s="13"/>
     </row>
-    <row r="4" spans="1:9" ht="64">
+    <row r="4" spans="1:9">
       <c r="A4" s="17"/>
       <c r="B4" s="17"/>
-      <c r="C4" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="11"/>
       <c r="E4" s="8"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" s="13" t="s">
-        <v>24</v>
-      </c>
+      <c r="H4" s="12"/>
+      <c r="I4" s="13"/>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="5"/>
@@ -754,47 +667,29 @@
       <c r="H5" s="14"/>
       <c r="I5" s="4"/>
     </row>
-    <row r="6" spans="1:9" ht="64">
+    <row r="6" spans="1:9">
       <c r="A6" s="15">
         <v>1</v>
       </c>
-      <c r="B6" s="15">
-        <v>2</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>17</v>
-      </c>
+      <c r="B6" s="15"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="10"/>
       <c r="E6" s="8"/>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
-      <c r="H6" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I6" s="13" t="s">
-        <v>24</v>
-      </c>
+      <c r="H6" s="12"/>
+      <c r="I6" s="13"/>
     </row>
-    <row r="7" spans="1:9" ht="48">
+    <row r="7" spans="1:9">
       <c r="A7" s="16"/>
       <c r="B7" s="16"/>
-      <c r="C7" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>18</v>
-      </c>
+      <c r="C7" s="6"/>
+      <c r="D7" s="10"/>
       <c r="E7" s="8"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
-      <c r="H7" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" s="13" t="s">
-        <v>24</v>
-      </c>
+      <c r="H7" s="12"/>
+      <c r="I7" s="13"/>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="17"/>

</xml_diff>